<commit_message>
feat: implement API key generation and storage functionality, update README and templates
</commit_message>
<xml_diff>
--- a/Appscripts/templates/Zendesk_Import_Assistant_Template.xlsx
+++ b/Appscripts/templates/Zendesk_Import_Assistant_Template.xlsx
@@ -14,7 +14,8 @@
     <sheet name="Validation Log" sheetId="10" r:id="rId10"/>
     <sheet name="Approval Log" sheetId="11" r:id="rId11"/>
     <sheet name="Execution Log" sheetId="12" r:id="rId12"/>
-    <sheet name="Schema Registry" sheetId="13" r:id="rId13"/>
+    <sheet name="Integration Secrets" sheetId="13" r:id="rId13"/>
+    <sheet name="Schema Registry" sheetId="14" r:id="rId14"/>
   </sheets>
 </workbook>
 </file>
@@ -200,6 +201,47 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>key_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>key_value</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>generated_at</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>generated_by</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>is_active</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Add progress narrator benchmarks and results, implement operating model benchmark, and enhance testing suite
- Introduced new benchmark results for progress narrator with detailed summaries and recommendations.
- Added JSON results for progress narrator benchmarks to capture detailed metrics.
- Created scripts to run operating model and progress narrator benchmarks.
- Developed comprehensive test cases for operating model and progress narrator functionalities.
- Implemented tests for Gemini client interactions and usage telemetry reporting.
- Enhanced frontend tests for the PreviewWorkspace component to ensure proper deployment phase handling.
</commit_message>
<xml_diff>
--- a/Appscripts/templates/Zendesk_Import_Assistant_Template.xlsx
+++ b/Appscripts/templates/Zendesk_Import_Assistant_Template.xlsx
@@ -6,16 +6,24 @@
     <sheet name="Planning Output" sheetId="2" r:id="rId2"/>
     <sheet name="Ticket Fields" sheetId="3" r:id="rId3"/>
     <sheet name="Ticket Forms" sheetId="4" r:id="rId4"/>
-    <sheet name="Macros" sheetId="5" r:id="rId5"/>
-    <sheet name="Triggers" sheetId="6" r:id="rId6"/>
-    <sheet name="Views" sheetId="7" r:id="rId7"/>
-    <sheet name="Tag Dictionary" sheetId="8" r:id="rId8"/>
-    <sheet name="Recommendations" sheetId="9" r:id="rId9"/>
-    <sheet name="Validation Log" sheetId="10" r:id="rId10"/>
-    <sheet name="Approval Log" sheetId="11" r:id="rId11"/>
-    <sheet name="Execution Log" sheetId="12" r:id="rId12"/>
-    <sheet name="Integration Secrets" sheetId="13" r:id="rId13"/>
-    <sheet name="Schema Registry" sheetId="14" r:id="rId14"/>
+    <sheet name="Brands" sheetId="5" r:id="rId5"/>
+    <sheet name="Groups" sheetId="6" r:id="rId6"/>
+    <sheet name="Macros" sheetId="7" r:id="rId7"/>
+    <sheet name="Triggers" sheetId="8" r:id="rId8"/>
+    <sheet name="Automations" sheetId="9" r:id="rId9"/>
+    <sheet name="Views" sheetId="10" r:id="rId10"/>
+    <sheet name="Tag Dictionary" sheetId="11" r:id="rId11"/>
+    <sheet name="Recommendations" sheetId="12" r:id="rId12"/>
+    <sheet name="Categories" sheetId="13" r:id="rId13"/>
+    <sheet name="Sections" sheetId="14" r:id="rId14"/>
+    <sheet name="Articles" sheetId="15" r:id="rId15"/>
+    <sheet name="Batch Metadata" sheetId="16" r:id="rId16"/>
+    <sheet name="Progress Log" sheetId="17" r:id="rId17"/>
+    <sheet name="Validation Log" sheetId="18" r:id="rId18"/>
+    <sheet name="Approval Log" sheetId="19" r:id="rId19"/>
+    <sheet name="Execution Log" sheetId="20" r:id="rId20"/>
+    <sheet name="Integration Secrets" sheetId="21" r:id="rId21"/>
+    <sheet name="Schema Registry" sheetId="22" r:id="rId22"/>
   </sheets>
 </workbook>
 </file>
@@ -63,6 +71,839 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:U1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>batch_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>object_type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>preview_summary</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>conditions_json</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>actions_json</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>validation_status</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>warning_message</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>blocked_reason</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>import_decision</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>approved_by</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>approved_at</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>deployment_status</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>zendesk_object_id</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>chunk_id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>record_key</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>source_provider</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>source_model</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:U1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>batch_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>object_type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>preview_summary</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>conditions_json</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>actions_json</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>validation_status</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>warning_message</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>blocked_reason</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>import_decision</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>approved_by</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>approved_at</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>deployment_status</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>zendesk_object_id</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>chunk_id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>record_key</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>source_provider</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>source_model</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:U1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>batch_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>object_type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>preview_summary</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>conditions_json</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>actions_json</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>validation_status</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>warning_message</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>blocked_reason</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>import_decision</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>approved_by</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>approved_at</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>deployment_status</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>zendesk_object_id</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>chunk_id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>record_key</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>source_provider</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>source_model</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:U1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>batch_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>object_type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>preview_summary</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>conditions_json</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>actions_json</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>validation_status</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>warning_message</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>blocked_reason</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>import_decision</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>approved_by</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>approved_at</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>deployment_status</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>zendesk_object_id</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>chunk_id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>record_key</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>source_provider</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>source_model</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:U1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>batch_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>object_type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>preview_summary</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>conditions_json</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>actions_json</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>validation_status</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>warning_message</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>blocked_reason</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>import_decision</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>approved_by</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>approved_at</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>deployment_status</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>zendesk_object_id</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>chunk_id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>record_key</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>source_provider</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>source_model</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:U1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>batch_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>object_type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>preview_summary</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>conditions_json</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>actions_json</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>validation_status</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>warning_message</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>blocked_reason</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>import_decision</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>approved_by</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>approved_at</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>deployment_status</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>zendesk_object_id</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>chunk_id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>record_key</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>source_provider</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>source_model</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>batch_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>coverage_status</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>coverage_manifest_json</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>department_coverage_json</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>quality_gates_json</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>supervisor_json</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>llm_routes_json</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>usage_report_json</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>orchestration_json</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>progress_narration_json</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>batch_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>wave</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>object_type</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>provider</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -112,7 +953,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -148,7 +989,38 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>batch_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>object_type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>intent</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -199,7 +1071,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -240,7 +1112,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -276,9 +1148,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D1"/>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:U1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -289,27 +1161,112 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>object_type</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>intent</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>confidence</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O1"/>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>preview_summary</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>conditions_json</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>actions_json</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>validation_status</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>warning_message</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>blocked_reason</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>import_decision</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>approved_by</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>approved_at</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>deployment_status</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>zendesk_object_id</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>chunk_id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>record_key</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>source_provider</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>source_model</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:U1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -388,14 +1345,44 @@
           <t>zendesk_object_id</t>
         </is>
       </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O1"/>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>chunk_id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>record_key</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>source_provider</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>source_model</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:U1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,14 +1461,44 @@
           <t>zendesk_object_id</t>
         </is>
       </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O1"/>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>chunk_id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>record_key</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>source_provider</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>source_model</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:U1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,14 +1577,44 @@
           <t>zendesk_object_id</t>
         </is>
       </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O1"/>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>chunk_id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>record_key</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>source_provider</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>source_model</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:U1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -646,14 +1693,44 @@
           <t>zendesk_object_id</t>
         </is>
       </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O1"/>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>chunk_id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>record_key</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>source_provider</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>source_model</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:U1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -732,14 +1809,44 @@
           <t>zendesk_object_id</t>
         </is>
       </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O1"/>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>chunk_id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>record_key</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>source_provider</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>source_model</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:U1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,90 +1925,34 @@
           <t>zendesk_object_id</t>
         </is>
       </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>batch_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>record_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>object_type</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>preview_summary</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>conditions_json</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>actions_json</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>validation_status</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>warning_message</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>blocked_reason</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>import_decision</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>approved_by</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>approved_at</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>deployment_status</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>zendesk_object_id</t>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>chunk_id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>record_key</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>source_provider</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>source_model</t>
         </is>
       </c>
     </row>

</xml_diff>